<commit_message>
add the extra excel file for distribution code ad erd file
</commit_message>
<xml_diff>
--- a/데이터 모델링1.xlsx
+++ b/데이터 모델링1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51E38C32-2249-469D-88E8-812DEE42A228}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03E8282D-44DD-4099-AD8F-806AF05F188F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1695" yWindow="2025" windowWidth="13485" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="150">
   <si>
     <t xml:space="preserve">User </t>
   </si>
@@ -158,9 +158,6 @@
     <t>행사 ID</t>
   </si>
   <si>
-    <t>FK (Event.event_id)</t>
-  </si>
-  <si>
     <t xml:space="preserve">추천 코스 </t>
   </si>
   <si>
@@ -464,55 +461,72 @@
     <t>sub_event</t>
   </si>
   <si>
+    <t>sponsor1</t>
+  </si>
+  <si>
+    <t>주최자</t>
+  </si>
+  <si>
+    <t>sponsor1_tel</t>
+  </si>
+  <si>
+    <t>주최자 연락처</t>
+  </si>
+  <si>
+    <t>sponsor2</t>
+  </si>
+  <si>
+    <t>주관자</t>
+  </si>
+  <si>
+    <t>sponsor2_tel</t>
+  </si>
+  <si>
+    <t>주관자 연락처</t>
+  </si>
+  <si>
+    <t>course_title</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>description</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
     <t>부대 행사</t>
-  </si>
-  <si>
-    <t>sponsor1</t>
-  </si>
-  <si>
-    <t>주최자</t>
-  </si>
-  <si>
-    <t>sponsor1_tel</t>
-  </si>
-  <si>
-    <t>주최자 연락처</t>
-  </si>
-  <si>
-    <t>sponsor2</t>
-  </si>
-  <si>
-    <t>주관자</t>
-  </si>
-  <si>
-    <t>sponsor2_tel</t>
-  </si>
-  <si>
-    <t>주관자 연락처</t>
-  </si>
-  <si>
-    <t>course_title</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>description</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>order</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>DEFA+C91:D106ULT CURRENT_TIMESTAMP</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>sequence</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>FK (Event.content_id)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -702,55 +716,58 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1298,8 +1315,8 @@
       <c r="C18" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>35</v>
+      <c r="D18" s="19" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1336,7 +1353,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -1358,13 +1375,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>8</v>
@@ -1386,13 +1403,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="C27" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>41</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>16</v>
@@ -1400,25 +1417,25 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="18" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D28" s="4"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="18" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B29" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>44</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>45</v>
       </c>
       <c r="D29" s="4"/>
     </row>
@@ -1438,25 +1455,25 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B31" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="C31" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>48</v>
       </c>
       <c r="D31" s="4"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B32" s="7" t="s">
         <v>18</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D32" s="7"/>
     </row>
@@ -1480,7 +1497,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -1502,13 +1519,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>8</v>
@@ -1516,16 +1533,16 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
@@ -1539,18 +1556,18 @@
         <v>34</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="19" t="s">
+      <c r="A41" s="20" t="s">
         <v>148</v>
       </c>
       <c r="B41" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D41" s="7" t="s">
         <v>16</v>
@@ -1570,7 +1587,7 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
@@ -1592,13 +1609,13 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>8</v>
@@ -1629,7 +1646,7 @@
         <v>34</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
@@ -1666,7 +1683,7 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -1694,21 +1711,21 @@
         <v>6</v>
       </c>
       <c r="C55" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D55" s="4" t="s">
         <v>61</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>16</v>
@@ -1716,13 +1733,13 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>16</v>
@@ -1730,61 +1747,61 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D58" s="4"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D59" s="4"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B60" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B60" s="4" t="s">
-        <v>40</v>
-      </c>
       <c r="C60" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D60" s="4"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C61" s="4" t="s">
         <v>71</v>
-      </c>
-      <c r="B61" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C61" s="4" t="s">
-        <v>72</v>
       </c>
       <c r="D61" s="4"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C62" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="B62" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C62" s="4" t="s">
-        <v>74</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>16</v>
@@ -1792,13 +1809,13 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C63" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="B63" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C63" s="4" t="s">
-        <v>76</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>16</v>
@@ -1806,100 +1823,100 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D64" s="4"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B65" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B65" s="4" t="s">
+      <c r="C65" s="4" t="s">
         <v>80</v>
-      </c>
-      <c r="C65" s="4" t="s">
-        <v>81</v>
       </c>
       <c r="D65" s="4"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C66" s="4" t="s">
         <v>82</v>
-      </c>
-      <c r="B66" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C66" s="4" t="s">
-        <v>83</v>
       </c>
       <c r="D66" s="4"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B67" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="C67" s="4" t="s">
         <v>85</v>
-      </c>
-      <c r="C67" s="4" t="s">
-        <v>86</v>
       </c>
       <c r="D67" s="4"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C68" s="4" t="s">
         <v>87</v>
-      </c>
-      <c r="B68" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C68" s="4" t="s">
-        <v>88</v>
       </c>
       <c r="D68" s="4"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C69" s="4" t="s">
         <v>89</v>
-      </c>
-      <c r="B69" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C69" s="4" t="s">
-        <v>90</v>
       </c>
       <c r="D69" s="4"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D70" s="4"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C71" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D71" s="4" t="s">
         <v>94</v>
-      </c>
-      <c r="D71" s="4" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
@@ -1910,7 +1927,7 @@
         <v>21</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>23</v>
@@ -1918,16 +1935,16 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B73" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="74" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1938,7 +1955,7 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
@@ -1960,13 +1977,13 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>8</v>
@@ -1980,10 +1997,10 @@
         <v>6</v>
       </c>
       <c r="C78" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D78" s="4" t="s">
         <v>102</v>
-      </c>
-      <c r="D78" s="4" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
@@ -1997,18 +2014,18 @@
         <v>34</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C80" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="B80" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C80" s="4" t="s">
-        <v>106</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>16</v>
@@ -2016,13 +2033,13 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B81" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D81" s="4" t="s">
         <v>16</v>
@@ -2036,7 +2053,7 @@
         <v>21</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>23</v>
@@ -2044,13 +2061,13 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>23</v>
@@ -2076,7 +2093,7 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
@@ -2098,13 +2115,13 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D89" s="4" t="s">
         <v>8</v>
@@ -2115,180 +2132,180 @@
         <v>33</v>
       </c>
       <c r="B90" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C90" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="C90" s="4" t="s">
+      <c r="D90" s="4" t="s">
         <v>116</v>
-      </c>
-      <c r="D90" s="4" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D91" s="4"/>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C92" s="4" t="s">
         <v>120</v>
-      </c>
-      <c r="B92" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C92" s="4" t="s">
-        <v>121</v>
       </c>
       <c r="D92" s="4"/>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B93" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D93" s="4"/>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D94" s="4"/>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B95" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D95" s="4"/>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D96" s="4"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B97" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D97" s="4"/>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C98" s="4" t="s">
         <v>132</v>
-      </c>
-      <c r="B98" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C98" s="4" t="s">
-        <v>133</v>
       </c>
       <c r="D98" s="4"/>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C99" s="4" t="s">
         <v>134</v>
-      </c>
-      <c r="B99" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C99" s="4" t="s">
-        <v>135</v>
       </c>
       <c r="D99" s="4"/>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C100" s="4" t="s">
-        <v>137</v>
+        <v>43</v>
+      </c>
+      <c r="C100" s="19" t="s">
+        <v>146</v>
       </c>
       <c r="D100" s="4"/>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" s="4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B101" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D101" s="4"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B102" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D102" s="4"/>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B103" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D103" s="4"/>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" s="4" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B104" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D104" s="4"/>
     </row>
@@ -2308,16 +2325,16 @@
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B106" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>23</v>
+        <v>147</v>
       </c>
     </row>
     <row r="107" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2327,7 +2344,7 @@
       <c r="D107" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>